<commit_message>
Fill unit price, drop statutory welfare row in 就労月報
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UcFZabuQnYW69BqxyN3p7g
</commit_message>
<xml_diff>
--- a/就労月報_スウェーデン大使館.xlsx
+++ b/就労月報_スウェーデン大使館.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,12 +35,8 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
-    <font>
-      <color rgb="00C00000"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -50,11 +46,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,13 +67,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -95,9 +85,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -469,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -507,225 +495,188 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>【記入方法】黄色セル（単価・法定福利費率）を入力すると金額が自動計算されます。</t>
-        </is>
-      </c>
-    </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>計</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>単位</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>単価</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>金額</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>金</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>土</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>月</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>火</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>水</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>木</t>
         </is>
       </c>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="4" t="n"/>
-      <c r="L6" s="7" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>作業員（昼間）</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>解体工</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n">
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="8">
         <f>SUM(B7:H7)</f>
         <v/>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>人工</t>
         </is>
       </c>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="11">
+      <c r="K7" s="9" t="n">
+        <v>33600</v>
+      </c>
+      <c r="L7" s="9">
         <f>IF(K7="","",I7*K7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>法定福利費</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>諸経費</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>率</t>
         </is>
       </c>
-      <c r="K8" s="12" t="n"/>
-      <c r="L8" s="11">
-        <f>IF(OR(K8="",L7=""),"",ROUND(L7*K8,0))</f>
+      <c r="K8" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="L8" s="9">
+        <f>IF(L7="","",ROUND(L7*K8,0))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>諸経費</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="inlineStr">
-        <is>
-          <t>率</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="L9" s="11">
-        <f>IF(L7="","",ROUND(L7*K9,0))</f>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>合　計（税抜）</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="13">
+        <f>SUM(L7:L8)</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>合　計（税抜）</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="15" t="n"/>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="15" t="n"/>
-      <c r="J10" s="15" t="n"/>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="16">
-        <f>SUM(L7:L9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>※道具代は含みません。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>※法定福利費・諸経費は人工金額にかけて計算。</t>
         </is>
       </c>
     </row>

</xml_diff>